<commit_message>
Added script to create documents and references
</commit_message>
<xml_diff>
--- a/template sheets/product specific configs/Documents and References Template.xlsx
+++ b/template sheets/product specific configs/Documents and References Template.xlsx
@@ -5,17 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kochind-my.sharepoint.com/personal/arjun_saravanakumar_molex_com/Documents/Desktop/Data Prep/MX150 2X10 RCPT (33472)/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kochind-my.sharepoint.com/personal/arjun_saravanakumar_molex_com/Documents/Desktop/Data Prep Automations/template sheets/product specific configs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="53" documentId="11_F25DC773A252ABDACC1048B4D9DF4EDC5ADE5902" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A058330-C0D5-4549-AF56-F7A113A377CD}"/>
+  <xr:revisionPtr revIDLastSave="59" documentId="11_F25DC773A252ABDACC1048B4D9DF4EDC5ADE5902" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91949F8A-5C9E-494A-9DB4-8DA3A4D05EAC}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="162913" refMode="R1C1" iterateCount="0" calcOnSave="0" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,63 +25,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
-    <t>Product</t>
+    <t>Product Name</t>
   </si>
   <si>
-    <t>Doc Type</t>
+    <t>Document type</t>
   </si>
   <si>
-    <t>Document Number</t>
+    <t>Document</t>
   </si>
   <si>
-    <t>PDD</t>
-  </si>
-  <si>
-    <t>PS</t>
-  </si>
-  <si>
-    <t>PSD</t>
-  </si>
-  <si>
-    <t>Document Part Number</t>
-  </si>
-  <si>
-    <t>E-33472-0002</t>
-  </si>
-  <si>
-    <t>PK-31300-903</t>
-  </si>
-  <si>
-    <t>AS-33472-100</t>
-  </si>
-  <si>
-    <t>AS-33611-001</t>
-  </si>
-  <si>
-    <t>PS-33472-000</t>
-  </si>
-  <si>
-    <t>TS-33472-0001</t>
-  </si>
-  <si>
-    <t>6L3T-14A464-AA</t>
-  </si>
-  <si>
-    <t>SD-33472-0001</t>
-  </si>
-  <si>
-    <t>SD-33472-0002</t>
-  </si>
-  <si>
-    <t>001</t>
-  </si>
-  <si>
-    <t>002</t>
-  </si>
-  <si>
-    <t>MX150 2X10 RCPT (33472)</t>
+    <t>Document Part</t>
   </si>
 </sst>
 </file>
@@ -437,7 +392,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.44140625" bestFit="1" customWidth="1"/>
   </cols>
@@ -453,134 +408,62 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>16</v>
-      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="4"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>16</v>
-      </c>
+      <c r="A3" s="2"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="4"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>16</v>
-      </c>
+      <c r="A4" s="2"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="4"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>16</v>
-      </c>
+      <c r="A5" s="2"/>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="4"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>16</v>
-      </c>
+      <c r="A6" s="2"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="4"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>16</v>
-      </c>
+      <c r="A7" s="2"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="4"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>16</v>
-      </c>
+      <c r="A8" s="2"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="4"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>16</v>
-      </c>
+      <c r="A9" s="2"/>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="4"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>17</v>
-      </c>
+      <c r="A10" s="2"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>

</xml_diff>